<commit_message>
Level 5: the four heroes' weapons reel (in progress): pilot way heroes and its runs
815 with level 5 and the way heroes (run5h): the Warrior, Mage, Warlock and Rogue each with the same session seed, so
the great hall's chests hold the same weapons for all four and the rules of who wields what show (armour refused, the
Mage's spells and mana potion, a short sword fought until it breaks, the Rogue's short blades and bow). Records in
cine_quartet_<hero>.json; the overlay, the menu pilot and the assembler follow. Not rendered to renders/ yet.
.gitignore: Blender build console logs and the pilot's rehearsal record. docs/levelups.xlsx updated.
</commit_message>
<xml_diff>
--- a/docs/levelups.xlsx
+++ b/docs/levelups.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="220">
   <si>
     <t>viking shortsword</t>
   </si>
@@ -655,6 +655,27 @@
   </si>
   <si>
     <t>up to 6 items can be found in any container.</t>
+  </si>
+  <si>
+    <t>tier 2 rooms</t>
+  </si>
+  <si>
+    <t>tier  1 rooms</t>
+  </si>
+  <si>
+    <t>tier 5 rooms</t>
+  </si>
+  <si>
+    <t>tier 3 rooms</t>
+  </si>
+  <si>
+    <t>tier 4 rooms</t>
+  </si>
+  <si>
+    <t>tier 4, 5 rooms</t>
+  </si>
+  <si>
+    <t>location</t>
   </si>
 </sst>
 </file>
@@ -1085,6 +1106,9 @@
       <c r="E3">
         <v>4</v>
       </c>
+      <c r="F3" t="s">
+        <v>205</v>
+      </c>
       <c r="G3">
         <v>68</v>
       </c>
@@ -1105,6 +1129,9 @@
       <c r="E4">
         <v>5</v>
       </c>
+      <c r="F4" t="s">
+        <v>213</v>
+      </c>
       <c r="G4">
         <v>69</v>
       </c>
@@ -1125,6 +1152,9 @@
       <c r="E5">
         <v>6</v>
       </c>
+      <c r="F5" t="s">
+        <v>213</v>
+      </c>
       <c r="G5">
         <v>70</v>
       </c>
@@ -1168,6 +1198,9 @@
       <c r="E7">
         <v>7</v>
       </c>
+      <c r="F7" t="s">
+        <v>205</v>
+      </c>
       <c r="G7">
         <v>87</v>
       </c>
@@ -1188,6 +1221,9 @@
       <c r="E8">
         <v>7</v>
       </c>
+      <c r="F8" t="s">
+        <v>214</v>
+      </c>
       <c r="G8">
         <v>88</v>
       </c>
@@ -1208,6 +1244,9 @@
       <c r="E9">
         <v>8</v>
       </c>
+      <c r="F9" t="s">
+        <v>213</v>
+      </c>
       <c r="G9">
         <v>89</v>
       </c>
@@ -1228,6 +1267,9 @@
       <c r="E10">
         <v>8</v>
       </c>
+      <c r="F10" t="s">
+        <v>213</v>
+      </c>
       <c r="G10">
         <v>90</v>
       </c>
@@ -1271,6 +1313,9 @@
       <c r="E12">
         <v>9</v>
       </c>
+      <c r="F12" t="s">
+        <v>213</v>
+      </c>
       <c r="G12">
         <v>98</v>
       </c>
@@ -1291,6 +1336,9 @@
       <c r="E13">
         <v>10</v>
       </c>
+      <c r="F13" t="s">
+        <v>216</v>
+      </c>
       <c r="G13">
         <v>99</v>
       </c>
@@ -1311,6 +1359,9 @@
       <c r="E14">
         <v>10</v>
       </c>
+      <c r="F14" t="s">
+        <v>218</v>
+      </c>
       <c r="G14">
         <v>100</v>
       </c>
@@ -1354,6 +1405,9 @@
       <c r="E16">
         <v>5</v>
       </c>
+      <c r="F16" t="s">
+        <v>213</v>
+      </c>
       <c r="G16">
         <v>79</v>
       </c>
@@ -1374,6 +1428,9 @@
       <c r="E17">
         <v>6</v>
       </c>
+      <c r="F17" t="s">
+        <v>216</v>
+      </c>
       <c r="G17">
         <v>80</v>
       </c>
@@ -1417,6 +1474,9 @@
       <c r="E19">
         <v>1</v>
       </c>
+      <c r="F19" t="s">
+        <v>205</v>
+      </c>
       <c r="G19">
         <v>53</v>
       </c>
@@ -1437,6 +1497,9 @@
       <c r="E20">
         <v>1</v>
       </c>
+      <c r="F20" t="s">
+        <v>213</v>
+      </c>
       <c r="G20">
         <v>54</v>
       </c>
@@ -1457,6 +1520,9 @@
       <c r="E21">
         <v>2</v>
       </c>
+      <c r="F21" t="s">
+        <v>213</v>
+      </c>
       <c r="G21">
         <v>55</v>
       </c>
@@ -1477,6 +1543,9 @@
       <c r="E22">
         <v>2</v>
       </c>
+      <c r="F22" t="s">
+        <v>216</v>
+      </c>
       <c r="G22">
         <v>56</v>
       </c>
@@ -1497,6 +1566,9 @@
       <c r="E23">
         <v>2</v>
       </c>
+      <c r="F23" t="s">
+        <v>216</v>
+      </c>
       <c r="G23">
         <v>57</v>
       </c>
@@ -1517,6 +1589,9 @@
       <c r="E24">
         <v>3</v>
       </c>
+      <c r="F24" t="s">
+        <v>217</v>
+      </c>
       <c r="G24">
         <v>58</v>
       </c>
@@ -1537,6 +1612,9 @@
       <c r="E25">
         <v>3</v>
       </c>
+      <c r="F25" t="s">
+        <v>217</v>
+      </c>
       <c r="G25">
         <v>59</v>
       </c>
@@ -1557,6 +1635,9 @@
       <c r="E26">
         <v>3</v>
       </c>
+      <c r="F26" t="s">
+        <v>215</v>
+      </c>
       <c r="G26">
         <v>60</v>
       </c>
@@ -1577,6 +1658,9 @@
       <c r="E27">
         <v>4</v>
       </c>
+      <c r="F27" t="s">
+        <v>205</v>
+      </c>
       <c r="G27">
         <v>72</v>
       </c>
@@ -1597,6 +1681,9 @@
       <c r="E28">
         <v>4</v>
       </c>
+      <c r="F28" t="s">
+        <v>213</v>
+      </c>
       <c r="G28">
         <v>73</v>
       </c>
@@ -1617,6 +1704,9 @@
       <c r="E29">
         <v>5</v>
       </c>
+      <c r="F29" t="s">
+        <v>216</v>
+      </c>
       <c r="G29">
         <v>74</v>
       </c>
@@ -1636,6 +1726,9 @@
       </c>
       <c r="E30">
         <v>6</v>
+      </c>
+      <c r="F30" t="s">
+        <v>218</v>
       </c>
       <c r="G30">
         <v>75</v>
@@ -1691,7 +1784,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="22.06640625" customWidth="1"/>
@@ -1699,9 +1792,10 @@
     <col min="3" max="3" width="22.9296875" customWidth="1"/>
     <col min="4" max="4" width="19.6640625" customWidth="1"/>
     <col min="5" max="5" width="18.265625" customWidth="1"/>
+    <col min="6" max="6" width="19.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
@@ -1717,8 +1811,11 @@
       <c r="E1" s="1" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F1" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -1734,8 +1831,11 @@
       <c r="E2">
         <v>510</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F2" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>41</v>
       </c>
@@ -1751,8 +1851,11 @@
       <c r="E3">
         <v>525</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F3" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>42</v>
       </c>
@@ -1768,8 +1871,11 @@
       <c r="E4">
         <v>525</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F4" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -1785,8 +1891,11 @@
       <c r="E5">
         <v>550</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F5" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>44</v>
       </c>
@@ -1802,8 +1911,11 @@
       <c r="E6">
         <v>575</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F6" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>45</v>
       </c>
@@ -1819,8 +1931,11 @@
       <c r="E7">
         <v>600</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F7" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>46</v>
       </c>
@@ -1836,8 +1951,11 @@
       <c r="E8">
         <v>600</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F8" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>48</v>
       </c>
@@ -1853,8 +1971,11 @@
       <c r="E9">
         <v>475</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F9" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>51</v>
       </c>
@@ -1870,8 +1991,11 @@
       <c r="E10">
         <v>500</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F10" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>50</v>
       </c>
@@ -1887,8 +2011,11 @@
       <c r="E11">
         <v>400</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F11" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>52</v>
       </c>
@@ -1904,8 +2031,11 @@
       <c r="E12">
         <v>375</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F12" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>54</v>
       </c>
@@ -1921,8 +2051,11 @@
       <c r="E13">
         <v>200</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F13" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>56</v>
       </c>
@@ -1938,8 +2071,11 @@
       <c r="E14">
         <v>175</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F14" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>57</v>
       </c>
@@ -1955,8 +2091,11 @@
       <c r="E15">
         <v>150</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F15" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>58</v>
       </c>
@@ -1972,8 +2111,11 @@
       <c r="E16">
         <v>210</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F16" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>59</v>
       </c>
@@ -1989,8 +2131,11 @@
       <c r="E17">
         <v>225</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F17" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>60</v>
       </c>
@@ -2006,8 +2151,11 @@
       <c r="E18">
         <v>250</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F18" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>61</v>
       </c>
@@ -2023,8 +2171,11 @@
       <c r="E19">
         <v>275</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F19" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>62</v>
       </c>
@@ -2040,8 +2191,11 @@
       <c r="E20">
         <v>300</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F20" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>64</v>
       </c>
@@ -2057,8 +2211,11 @@
       <c r="E21">
         <v>125</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F21" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>65</v>
       </c>
@@ -2074,8 +2231,11 @@
       <c r="E22">
         <v>150</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F22" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>66</v>
       </c>
@@ -2091,8 +2251,11 @@
       <c r="E23">
         <v>175</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F23" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>67</v>
       </c>
@@ -2108,8 +2271,11 @@
       <c r="E24">
         <v>200</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F24" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>68</v>
       </c>
@@ -2125,8 +2291,11 @@
       <c r="E25">
         <v>375</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F25" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>69</v>
       </c>
@@ -2142,8 +2311,11 @@
       <c r="E26">
         <v>400</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F26" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>70</v>
       </c>
@@ -2159,8 +2331,11 @@
       <c r="E27">
         <v>475</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F27" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>71</v>
       </c>
@@ -2176,8 +2351,11 @@
       <c r="E28">
         <v>510</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F28" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>75</v>
       </c>
@@ -2185,7 +2363,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>78</v>
       </c>
@@ -2250,6 +2428,9 @@
         <v>0.1</v>
       </c>
       <c r="C3" s="2"/>
+      <c r="G3" t="s">
+        <v>205</v>
+      </c>
       <c r="H3" s="2">
         <v>0.8</v>
       </c>
@@ -2262,6 +2443,9 @@
         <v>0.2</v>
       </c>
       <c r="C4" s="2"/>
+      <c r="G4" t="s">
+        <v>205</v>
+      </c>
       <c r="H4" s="2">
         <v>0.7</v>
       </c>
@@ -2274,6 +2458,9 @@
         <v>0.3</v>
       </c>
       <c r="C5" s="2"/>
+      <c r="G5" t="s">
+        <v>213</v>
+      </c>
       <c r="H5" s="2">
         <v>0.6</v>
       </c>
@@ -2286,6 +2473,9 @@
         <v>0.4</v>
       </c>
       <c r="C6" s="2"/>
+      <c r="G6" t="s">
+        <v>213</v>
+      </c>
       <c r="H6" s="2">
         <v>0.5</v>
       </c>
@@ -2298,6 +2488,9 @@
         <v>0.5</v>
       </c>
       <c r="C7" s="2"/>
+      <c r="G7" t="s">
+        <v>216</v>
+      </c>
       <c r="H7" s="2">
         <v>0.4</v>
       </c>
@@ -2310,6 +2503,9 @@
         <v>0.6</v>
       </c>
       <c r="C8" s="2"/>
+      <c r="G8" t="s">
+        <v>216</v>
+      </c>
       <c r="H8" s="2">
         <v>0.3</v>
       </c>
@@ -2322,6 +2518,9 @@
         <v>0.7</v>
       </c>
       <c r="C9" s="2"/>
+      <c r="G9" t="s">
+        <v>217</v>
+      </c>
       <c r="H9" s="2">
         <v>0.2</v>
       </c>
@@ -2334,6 +2533,9 @@
         <v>0.8</v>
       </c>
       <c r="C10" s="2"/>
+      <c r="G10" t="s">
+        <v>215</v>
+      </c>
       <c r="H10" s="2">
         <v>0.1</v>
       </c>
@@ -2345,6 +2547,9 @@
       <c r="C11" s="2">
         <v>0.1</v>
       </c>
+      <c r="G11" t="s">
+        <v>205</v>
+      </c>
       <c r="H11" s="2">
         <v>0.8</v>
       </c>
@@ -2356,6 +2561,9 @@
       <c r="C12" s="2">
         <v>0.2</v>
       </c>
+      <c r="G12" t="s">
+        <v>205</v>
+      </c>
       <c r="H12" s="2">
         <v>0.7</v>
       </c>
@@ -2367,6 +2575,9 @@
       <c r="C13" s="2">
         <v>0.3</v>
       </c>
+      <c r="G13" t="s">
+        <v>213</v>
+      </c>
       <c r="H13" s="2">
         <v>0.6</v>
       </c>
@@ -2378,6 +2589,9 @@
       <c r="C14" s="2">
         <v>0.4</v>
       </c>
+      <c r="G14" t="s">
+        <v>213</v>
+      </c>
       <c r="H14" s="2">
         <v>0.5</v>
       </c>
@@ -2389,6 +2603,9 @@
       <c r="C15" s="2">
         <v>0.5</v>
       </c>
+      <c r="G15" t="s">
+        <v>216</v>
+      </c>
       <c r="H15" s="2">
         <v>0.4</v>
       </c>
@@ -2400,6 +2617,9 @@
       <c r="C16" s="2">
         <v>0.6</v>
       </c>
+      <c r="G16" t="s">
+        <v>216</v>
+      </c>
       <c r="H16" s="2">
         <v>0.3</v>
       </c>
@@ -2411,6 +2631,9 @@
       <c r="C17" s="2">
         <v>0.7</v>
       </c>
+      <c r="G17" t="s">
+        <v>217</v>
+      </c>
       <c r="H17" s="2">
         <v>0.2</v>
       </c>
@@ -2422,6 +2645,9 @@
       <c r="C18" s="2">
         <v>0.8</v>
       </c>
+      <c r="G18" t="s">
+        <v>215</v>
+      </c>
       <c r="H18" s="2">
         <v>0.1</v>
       </c>
@@ -2433,6 +2659,9 @@
       <c r="E19" t="s">
         <v>126</v>
       </c>
+      <c r="G19" t="s">
+        <v>205</v>
+      </c>
       <c r="H19" s="2">
         <v>0.8</v>
       </c>
@@ -2444,6 +2673,9 @@
       <c r="E20" t="s">
         <v>127</v>
       </c>
+      <c r="G20" t="s">
+        <v>205</v>
+      </c>
       <c r="H20" s="2">
         <v>0.7</v>
       </c>
@@ -2455,6 +2687,9 @@
       <c r="E21" t="s">
         <v>128</v>
       </c>
+      <c r="G21" t="s">
+        <v>213</v>
+      </c>
       <c r="H21" s="2">
         <v>0.6</v>
       </c>
@@ -2466,6 +2701,9 @@
       <c r="E22" t="s">
         <v>129</v>
       </c>
+      <c r="G22" t="s">
+        <v>213</v>
+      </c>
       <c r="H22" s="2">
         <v>0.5</v>
       </c>
@@ -2477,6 +2715,9 @@
       <c r="E23" t="s">
         <v>130</v>
       </c>
+      <c r="G23" t="s">
+        <v>216</v>
+      </c>
       <c r="H23" s="2">
         <v>0.4</v>
       </c>
@@ -2488,6 +2729,9 @@
       <c r="E24" t="s">
         <v>131</v>
       </c>
+      <c r="G24" t="s">
+        <v>216</v>
+      </c>
       <c r="H24" s="2">
         <v>0.3</v>
       </c>
@@ -2499,6 +2743,9 @@
       <c r="E25" t="s">
         <v>132</v>
       </c>
+      <c r="G25" t="s">
+        <v>217</v>
+      </c>
       <c r="H25" s="2">
         <v>0.2</v>
       </c>
@@ -2510,6 +2757,9 @@
       <c r="E26" t="s">
         <v>133</v>
       </c>
+      <c r="G26" t="s">
+        <v>215</v>
+      </c>
       <c r="H26" s="2">
         <v>0.1</v>
       </c>
@@ -2521,6 +2771,9 @@
       <c r="D27" t="s">
         <v>109</v>
       </c>
+      <c r="G27" t="s">
+        <v>205</v>
+      </c>
       <c r="H27" s="2">
         <v>0.8</v>
       </c>
@@ -2532,6 +2785,9 @@
       <c r="D28" t="s">
         <v>110</v>
       </c>
+      <c r="G28" t="s">
+        <v>205</v>
+      </c>
       <c r="H28" s="2">
         <v>0.7</v>
       </c>
@@ -2543,6 +2799,9 @@
       <c r="D29" t="s">
         <v>111</v>
       </c>
+      <c r="G29" t="s">
+        <v>213</v>
+      </c>
       <c r="H29" s="2">
         <v>0.6</v>
       </c>
@@ -2554,6 +2813,9 @@
       <c r="D30" t="s">
         <v>112</v>
       </c>
+      <c r="G30" t="s">
+        <v>213</v>
+      </c>
       <c r="H30" s="2">
         <v>0.5</v>
       </c>
@@ -2565,6 +2827,9 @@
       <c r="D31" t="s">
         <v>113</v>
       </c>
+      <c r="G31" t="s">
+        <v>216</v>
+      </c>
       <c r="H31" s="2">
         <v>0.4</v>
       </c>
@@ -2576,6 +2841,9 @@
       <c r="D32" t="s">
         <v>114</v>
       </c>
+      <c r="G32" t="s">
+        <v>216</v>
+      </c>
       <c r="H32" s="2">
         <v>0.3</v>
       </c>
@@ -2587,6 +2855,9 @@
       <c r="D33" t="s">
         <v>115</v>
       </c>
+      <c r="G33" t="s">
+        <v>217</v>
+      </c>
       <c r="H33" s="2">
         <v>0.2</v>
       </c>
@@ -2598,6 +2869,9 @@
       <c r="D34" t="s">
         <v>116</v>
       </c>
+      <c r="G34" t="s">
+        <v>215</v>
+      </c>
       <c r="H34" s="2">
         <v>0.1</v>
       </c>
@@ -2609,6 +2883,9 @@
       <c r="D35" t="s">
         <v>117</v>
       </c>
+      <c r="G35" t="s">
+        <v>215</v>
+      </c>
       <c r="H35" s="2">
         <v>0.05</v>
       </c>
@@ -2620,6 +2897,9 @@
       <c r="F36" t="s">
         <v>157</v>
       </c>
+      <c r="G36" t="s">
+        <v>209</v>
+      </c>
       <c r="H36" s="2">
         <v>0.25</v>
       </c>
@@ -2631,6 +2911,9 @@
       <c r="F37" t="s">
         <v>157</v>
       </c>
+      <c r="G37" t="s">
+        <v>209</v>
+      </c>
       <c r="H37" s="2">
         <v>0.25</v>
       </c>
@@ -2642,6 +2925,9 @@
       <c r="F38" t="s">
         <v>157</v>
       </c>
+      <c r="G38" t="s">
+        <v>209</v>
+      </c>
       <c r="H38" s="2">
         <v>0.25</v>
       </c>
@@ -2653,6 +2939,9 @@
       <c r="F39" t="s">
         <v>157</v>
       </c>
+      <c r="G39" t="s">
+        <v>209</v>
+      </c>
       <c r="H39" s="2">
         <v>0.25</v>
       </c>
@@ -2664,6 +2953,9 @@
       <c r="F40" t="s">
         <v>157</v>
       </c>
+      <c r="G40" t="s">
+        <v>209</v>
+      </c>
       <c r="H40" s="2">
         <v>0.25</v>
       </c>
@@ -2675,6 +2967,9 @@
       <c r="F41" t="s">
         <v>157</v>
       </c>
+      <c r="G41" t="s">
+        <v>209</v>
+      </c>
       <c r="H41" s="2">
         <v>0.25</v>
       </c>
@@ -2686,6 +2981,9 @@
       <c r="F42" t="s">
         <v>157</v>
       </c>
+      <c r="G42" t="s">
+        <v>209</v>
+      </c>
       <c r="H42" s="2">
         <v>0.25</v>
       </c>
@@ -2697,6 +2995,9 @@
       <c r="F43" t="s">
         <v>157</v>
       </c>
+      <c r="G43" t="s">
+        <v>209</v>
+      </c>
       <c r="H43" s="2">
         <v>0.25</v>
       </c>
@@ -2708,6 +3009,9 @@
       <c r="F44" t="s">
         <v>157</v>
       </c>
+      <c r="G44" t="s">
+        <v>209</v>
+      </c>
       <c r="H44" s="2">
         <v>0.25</v>
       </c>
@@ -2719,6 +3023,9 @@
       <c r="F45" t="s">
         <v>157</v>
       </c>
+      <c r="G45" t="s">
+        <v>209</v>
+      </c>
       <c r="H45" s="2">
         <v>0.25</v>
       </c>
@@ -2730,6 +3037,9 @@
       <c r="F46" t="s">
         <v>157</v>
       </c>
+      <c r="G46" t="s">
+        <v>209</v>
+      </c>
       <c r="H46" s="2">
         <v>0.25</v>
       </c>
@@ -2741,6 +3051,9 @@
       <c r="F47" t="s">
         <v>157</v>
       </c>
+      <c r="G47" t="s">
+        <v>209</v>
+      </c>
       <c r="H47" s="2">
         <v>0.25</v>
       </c>
@@ -2752,6 +3065,9 @@
       <c r="F48" t="s">
         <v>157</v>
       </c>
+      <c r="G48" t="s">
+        <v>209</v>
+      </c>
       <c r="H48" s="2">
         <v>0.25</v>
       </c>
@@ -2763,6 +3079,9 @@
       <c r="F49" t="s">
         <v>157</v>
       </c>
+      <c r="G49" t="s">
+        <v>209</v>
+      </c>
       <c r="H49" s="2">
         <v>0.25</v>
       </c>
@@ -2773,6 +3092,9 @@
       </c>
       <c r="F50" t="s">
         <v>157</v>
+      </c>
+      <c r="G50" t="s">
+        <v>209</v>
       </c>
       <c r="H50" s="2">
         <v>0.25</v>

</xml_diff>